<commit_message>
KFSPTS-37934 add more changes for Register Asset extract
</commit_message>
<xml_diff>
--- a/src/main/resources/edu/cornell/kfs/cemi/module/cam/batch/Register_Asset.xlsx
+++ b/src/main/resources/edu/cornell/kfs/cemi/module/cam/batch/Register_Asset.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://huroncg.sharepoint.com/teams/edu/op/meth/Documents/Practice Area Methodologies/Higher Education/ES Cloud Methodology/4. Workday Implementation/Technical/Conversion/CloverDX Framework/CloverDX Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="414" documentId="8_{5EE89BE0-FDFB-4C44-BAEC-328D22962ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12539309-A3CD-4E97-BB44-803531072D2E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{234EE7B6-E6B9-4094-9ABC-11C4FF273C26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2449,7 +2449,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="161">
   <si>
     <t>Register Asset</t>
   </si>
@@ -2487,177 +2487,6 @@
   </si>
   <si>
     <t>Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Extract using legacy values:
-WCM: SAP - 8 digit Asset Number field
-Ithaca: KFS - 6 digit Asset Number field
-</t>
-  </si>
-  <si>
-    <t>use the same logic from column B</t>
-  </si>
-  <si>
-    <t>map to:
-C01 - statutory (contract colleges)
-C02 - endowed
-C03 - WCM NY
-C04 - WCM Qatar</t>
-  </si>
-  <si>
-    <t>WCM: Manufacturer field - only bring in Model values - determine with functional teams how to capture just the model information
-Ithaca: Model Number</t>
-  </si>
-  <si>
-    <t>WCM: Asset Description
-Ithaca: Asset Description</t>
-  </si>
-  <si>
-    <t>WCM: Use Asset Class to map to Spend Categories
-Ithaca: Use Asset Type/Object Code to map to existing Spend Categories in Workday - Nick to provide current list of Spend Category IDs</t>
-  </si>
-  <si>
-    <t>NON-DEPRECIABLE_CAPITAL_ASSET, CAPITALIZED, or EXPENSE
-WCM: If Asset Class 1000 = NON-DEPRECIABLE_CAPITAL_ASSET, ELSE CAPITALIZED
-Ithaca: Use Acquisition Type Name/Asset Type Name</t>
-  </si>
-  <si>
-    <t>WCM: LEASED when asset class is between 7000-7300
-Most others, default PURCHASED with few exceptions (Conversion team to work with Rosanna on exact logic)
-Equipment:
-If Asset is 32001475, 32001717 or 32002562, OTHER,
-If Asset Class is 7000 or 7300, LEASED,
-If Asset Class is between 2000-3600, PURCHASED
-Non Equipment:
-If Asset Class is 1300 or 1400, LEASED, else CONSTRUCTED (Asset # 45000283 = PURCHASED)
-Ithaca: Acquisition Type - use the following logic
-If GIK (Gift), Transfer (Transferred from other university or federal) and GFE = Other
-Purchased (New) = PURCHASED</t>
-  </si>
-  <si>
-    <t>WCM: leave blank for now (functional to confirm if data is needed here)
-Ithaca: Acquisition Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-WCM: S_ALR_87011990
-"Current APC"
-Ithaca: Asset Total Cost or Total Cost</t>
-  </si>
-  <si>
-    <t>Estimated amount at the end of the asset life
-WCM: leave blank
-Ithaca: Salvage Value</t>
-  </si>
-  <si>
-    <t>leave blank</t>
-  </si>
-  <si>
-    <t>WCM: default to 1
-Ithaca: default to 1</t>
-  </si>
-  <si>
-    <t>default to Cost_Center_ID</t>
-  </si>
-  <si>
-    <t>Nick to provide all cost center values - work with functional team to determine mapping
-WCM: Cost Center Ref ID
-Ithaca: Cost Center Ref ID</t>
-  </si>
-  <si>
-    <t>default to Fund_ID</t>
-  </si>
-  <si>
-    <t>Nick to provide all fund values - work with functional team to determine mapping
-WCM: Fund Ref ID
-Ithaca: Fund Ref ID</t>
-  </si>
-  <si>
-    <t>leave blank for now - will have to revisit and map Projects here</t>
-  </si>
-  <si>
-    <t>WCM: Capitalized On date
-Ithaca: Asset Create Date</t>
-  </si>
-  <si>
-    <t>WCM: Capitalized On date
-Ithaca: In Service Date</t>
-  </si>
-  <si>
-    <t>WCM: Weill_Cornell_New_York or Weill_Cornell_Qatar
-Ithaca: Cornell_University_Ithaca</t>
-  </si>
-  <si>
-    <t>WCM: Tag Number
-Ithaca: Tag Number</t>
-  </si>
-  <si>
-    <t>WCM: Serial Number
-Ithaca: Serial number</t>
-  </si>
-  <si>
-    <t>WCM: "Manufacturer of Asset"
-will need to be modified. Currently Manufacturer and Model are in one field - only pull the data prior to the /
-Ithaca: "Manfacturer" Many will need to be modified due to previous conversion errors - data cleanup will occur in legacy system, conversion team to extract as is.</t>
-  </si>
-  <si>
-    <t>Nick to provide reference ids from Workday
-WCM: Not currently tracked. Leave empty for now. 
-Ithaca: Asset Class ID in mapping file - Asset Type Code field</t>
-  </si>
-  <si>
-    <t>Valid Values - Noncapital, Equipment, Building, Land, Software
-WCM: Use the Asset Class. Will need cross walk for coded values out of SAP into Workday
-Ithaca: Asset Type ID in mapping file - Asset Object Sub Type</t>
-  </si>
-  <si>
-    <t>WCM: Inventory Note - need to work on mapping to Cost Center Ref ID in Workday
-Ithaca: Organization Owner Account Number - need to work on mapping to Cost Center Ref ID in Workday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Similar to Custodian. The worker responsible for the Asset.
-WCM: Responsible Party in SAP. Target employee ID. Expect some data load fallouts due to legacy employee IDs that may not have been updated after they left. 
-Ithaca: Asset Representative Name in KFS. Will need to net ID for employee id </t>
-  </si>
-  <si>
-    <t>WCM:  "Additional Inventory Description"
-will need to be modified. Currently PO Number and funding accounts (fund/WBS) are in one field
-Ithaca: Purchase Order Number</t>
-  </si>
-  <si>
-    <t>This isn't fully built out yet in Workday. 
-WCM: S_ALR_87011990. 
-field name: "Usefull Life" 
-Ithaca: Business to provide coded values for refrence to workday ID values. 
-field: Asset Type Codes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WCM: default to STRAIGHT_LINE
-Ithaca: default to STRAIGHT_LINE
-</t>
-  </si>
-  <si>
-    <t>Leave Blank</t>
-  </si>
-  <si>
-    <t>Required. Calculation based off of column AF. This is number of months. EX: if 10 years then 120 for 120 months. 
-WCM: see above
-Ithaca: see above</t>
-  </si>
-  <si>
-    <t>Gold build: Start of the fiscal year that we go-live in. 7/1 of the go-live year. 
-For Workset B: use 7/01/2026</t>
-  </si>
-  <si>
-    <t>WCM: Vi to work with business team to determine forumla/logic to capture remaining periods. 
-Ithaca: Vi to work with business team to determine forumla/logic to capture remaining periods.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WCM: S_ALR_87011990
-"Accumulated Depreciation"
-Ithaca: "Accumulated Depreciation"
-</t>
   </si>
   <si>
     <t>Area</t>
@@ -3792,131 +3621,55 @@
       <c r="AL1" s="9"/>
       <c r="AM1" s="9"/>
     </row>
-    <row r="2" spans="1:39" s="32" customFormat="1" ht="112.5" customHeight="1">
+    <row r="2" spans="1:39" s="32" customFormat="1" ht="84.75" customHeight="1">
       <c r="A2" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="29" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="29" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="29" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="29" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="29" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" s="29" t="s">
-        <v>16</v>
-      </c>
-      <c r="K2" s="30" t="s">
-        <v>17</v>
-      </c>
-      <c r="L2" s="30" t="s">
-        <v>18</v>
-      </c>
-      <c r="M2" s="30" t="s">
-        <v>19</v>
-      </c>
-      <c r="N2" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="O2" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="P2" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q2" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="R2" s="29" t="s">
-        <v>24</v>
-      </c>
-      <c r="S2" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="T2" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="U2" s="29" t="s">
-        <v>26</v>
-      </c>
-      <c r="V2" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="W2" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="X2" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="Y2" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="Z2" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="AA2" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB2" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC2" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="AD2" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE2" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="AF2" s="30" t="s">
-        <v>37</v>
-      </c>
-      <c r="AG2" s="30" t="s">
-        <v>38</v>
-      </c>
-      <c r="AH2" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="AI2" s="30" t="s">
-        <v>40</v>
-      </c>
-      <c r="AJ2" s="30" t="s">
-        <v>39</v>
-      </c>
-      <c r="AK2" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="AL2" s="30" t="s">
-        <v>42</v>
-      </c>
-      <c r="AM2" s="30" t="s">
-        <v>43</v>
-      </c>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
+      <c r="N2" s="30"/>
+      <c r="O2" s="29"/>
+      <c r="P2" s="29"/>
+      <c r="Q2" s="29"/>
+      <c r="R2" s="29"/>
+      <c r="S2" s="29"/>
+      <c r="T2" s="29"/>
+      <c r="U2" s="29"/>
+      <c r="V2" s="29"/>
+      <c r="W2" s="29"/>
+      <c r="X2" s="29"/>
+      <c r="Y2" s="29"/>
+      <c r="Z2" s="29"/>
+      <c r="AA2" s="29"/>
+      <c r="AB2" s="29"/>
+      <c r="AC2" s="29"/>
+      <c r="AD2" s="31"/>
+      <c r="AE2" s="30"/>
+      <c r="AF2" s="30"/>
+      <c r="AG2" s="30"/>
+      <c r="AH2" s="29"/>
+      <c r="AI2" s="30"/>
+      <c r="AJ2" s="30"/>
+      <c r="AK2" s="30"/>
+      <c r="AL2" s="30"/>
+      <c r="AM2" s="30"/>
     </row>
     <row r="3" spans="1:39" ht="18">
       <c r="A3" s="12" t="s">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="11"/>
@@ -3931,7 +3684,7 @@
       <c r="M3" s="11"/>
       <c r="N3" s="11"/>
       <c r="O3" s="16" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="P3" s="16"/>
       <c r="Q3" s="16"/>
@@ -3939,7 +3692,7 @@
       <c r="S3" s="16"/>
       <c r="T3" s="16"/>
       <c r="U3" s="11" t="s">
-        <v>47</v>
+        <v>11</v>
       </c>
       <c r="V3" s="11"/>
       <c r="W3" s="11"/>
@@ -3952,7 +3705,7 @@
       <c r="AD3" s="11"/>
       <c r="AE3" s="11"/>
       <c r="AF3" s="16" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="AG3" s="16"/>
       <c r="AH3" s="16"/>
@@ -3964,359 +3717,359 @@
     </row>
     <row r="4" spans="1:39" ht="18">
       <c r="A4" s="12" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="O4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="P4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="Q4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="S4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="T4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="U4" s="17" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="W4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="X4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="Y4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="AB4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="AC4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="AD4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="AE4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="AF4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="AG4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="AH4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="AI4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="AJ4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="AK4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AL4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AM4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:39" ht="18">
       <c r="A5" s="12" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>59</v>
+        <v>23</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="S5" s="1" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="T5" s="1" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="W5" s="1" t="s">
-        <v>65</v>
+        <v>29</v>
       </c>
       <c r="X5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="Y5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="AA5" s="1" t="s">
-        <v>66</v>
+        <v>30</v>
       </c>
       <c r="AB5" s="1" t="s">
-        <v>67</v>
+        <v>31</v>
       </c>
       <c r="AC5" s="1" t="s">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="AD5" s="1" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="AE5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="AF5" s="1" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="AG5" s="1" t="s">
-        <v>71</v>
+        <v>35</v>
       </c>
       <c r="AH5" s="1" t="s">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="AI5" s="1" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="AJ5" s="1" t="s">
-        <v>73</v>
+        <v>37</v>
       </c>
       <c r="AK5" s="1" t="s">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="AL5" s="1" t="s">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="AM5" s="1" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:39" ht="18">
       <c r="A6" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="L6" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="M6" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="N6" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="O6" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="P6" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q6" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="R6" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="S6" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="T6" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="U6" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="V6" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="W6" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="X6" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="Y6" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z6" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA6" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="AB6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC6" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="AD6" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="AE6" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="AF6" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="AG6" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH6" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="AI6" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="AJ6" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK6" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="AL6" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="AM6" s="11" t="s">
         <v>76</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="H6" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="I6" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="J6" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="K6" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="L6" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="M6" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="N6" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="O6" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="P6" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q6" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="R6" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="S6" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="T6" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="U6" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="V6" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="W6" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="X6" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="Y6" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="Z6" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="AA6" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="AB6" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="AC6" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="AD6" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="AE6" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="AF6" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="AG6" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="AH6" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="AI6" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="AJ6" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="AK6" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="AL6" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="AM6" s="11" t="s">
-        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -4463,10 +4216,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="F1" s="9"/>
       <c r="G1" s="9"/>
@@ -4529,7 +4282,7 @@
       <c r="BF1" s="9"/>
       <c r="BG1" s="9"/>
       <c r="BH1" s="9" t="s">
-        <v>114</v>
+        <v>78</v>
       </c>
       <c r="BI1" s="9"/>
       <c r="BJ1" s="9"/>
@@ -4561,7 +4314,7 @@
       <c r="BZ1" s="9"/>
       <c r="CA1" s="9"/>
       <c r="CB1" s="9" t="s">
-        <v>115</v>
+        <v>79</v>
       </c>
       <c r="CC1" s="9"/>
       <c r="CD1" s="9"/>
@@ -4654,10 +4407,10 @@
     </row>
     <row r="3" spans="1:82" ht="18">
       <c r="A3" s="12" t="s">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="11"/>
@@ -4675,7 +4428,7 @@
       <c r="P3" s="11"/>
       <c r="Q3" s="11"/>
       <c r="R3" s="16" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="S3" s="16"/>
       <c r="T3" s="16"/>
@@ -4689,61 +4442,61 @@
       <c r="AB3" s="16"/>
       <c r="AC3" s="16"/>
       <c r="AD3" s="19" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AE3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AF3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AG3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AH3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AI3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AJ3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AK3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AL3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AM3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AN3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AO3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AP3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AQ3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AR3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AS3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AT3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AU3" s="20" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="AV3" s="11" t="s">
-        <v>47</v>
+        <v>11</v>
       </c>
       <c r="AW3" s="11"/>
       <c r="AX3" s="11"/>
@@ -4768,7 +4521,7 @@
       <c r="BQ3" s="11"/>
       <c r="BR3" s="11"/>
       <c r="BS3" s="16" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="BT3" s="16"/>
       <c r="BU3" s="16"/>
@@ -4779,764 +4532,764 @@
       <c r="BZ3" s="16"/>
       <c r="CA3" s="16"/>
       <c r="CB3" s="11" t="s">
-        <v>117</v>
+        <v>81</v>
       </c>
       <c r="CC3" s="11"/>
       <c r="CD3" s="11"/>
     </row>
     <row r="4" spans="1:82" ht="18">
       <c r="A4" s="12" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="J4" s="17" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="L4" s="17" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="S4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="T4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="U4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="V4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="W4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="X4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="Y4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="Z4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AA4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AB4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AC4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AD4" s="21" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AE4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AF4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AG4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AH4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AI4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AJ4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AK4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AL4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AM4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AN4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AO4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AP4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AQ4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AR4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AS4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AT4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AU4" s="22" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="AV4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="AW4" s="17" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="AX4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="AY4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="AZ4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BA4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BB4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BC4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BD4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BE4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BF4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BG4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BH4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BI4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BJ4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BK4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BL4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BM4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BN4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BO4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BP4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BQ4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BR4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BS4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BT4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BU4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BV4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BW4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="BX4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="BY4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="BZ4" s="17" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="CA4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="CB4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="CC4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="CD4" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:82" ht="18">
       <c r="A5" s="12" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>118</v>
+        <v>82</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>118</v>
+        <v>82</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>119</v>
+        <v>83</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>59</v>
+        <v>23</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="S5" s="1" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="T5" s="1" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="W5" s="1" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="X5" s="1" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="Y5" s="1" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="AA5" s="1" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="AB5" s="1" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="AC5" s="1" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="AD5" s="23" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="AE5" s="24" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="AF5" s="24" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="AG5" s="24" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="AH5" s="24" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="AI5" s="24" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="AJ5" s="24" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="AK5" s="24" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="AL5" s="24" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="AM5" s="24" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="AN5" s="24" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="AO5" s="24" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="AP5" s="24" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="AQ5" s="24" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="AR5" s="24" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="AS5" s="24" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="AT5" s="24" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="AU5" s="24" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="AV5" s="1" t="s">
-        <v>120</v>
+        <v>84</v>
       </c>
       <c r="AW5" s="1" t="s">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="AX5" s="1" t="s">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="AY5" s="1" t="s">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="AZ5" s="1" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="BA5" s="1" t="s">
-        <v>121</v>
+        <v>85</v>
       </c>
       <c r="BB5" s="1" t="s">
-        <v>65</v>
+        <v>29</v>
       </c>
       <c r="BC5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="BD5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="BE5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="BF5" s="1" t="s">
-        <v>66</v>
+        <v>30</v>
       </c>
       <c r="BG5" s="1" t="s">
-        <v>67</v>
+        <v>31</v>
       </c>
       <c r="BH5" s="1" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="BI5" s="1" t="s">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="BJ5" s="1" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="BK5" s="1" t="s">
-        <v>122</v>
+        <v>86</v>
       </c>
       <c r="BL5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="BM5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="BN5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="BO5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="BP5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="BQ5" s="1" t="s">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="BR5" s="1" t="s">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="BS5" s="1" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="BT5" s="1" t="s">
-        <v>71</v>
+        <v>35</v>
       </c>
       <c r="BU5" s="1" t="s">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="BV5" s="1" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="BW5" s="1" t="s">
-        <v>73</v>
+        <v>37</v>
       </c>
       <c r="BX5" s="1" t="s">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="BY5" s="1" t="s">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="BZ5" s="1" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="CA5" s="1" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="CB5" s="1" t="s">
-        <v>118</v>
+        <v>82</v>
       </c>
       <c r="CC5" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="CD5" s="1" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:82" ht="18">
       <c r="A6" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="L6" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="M6" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="N6" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="O6" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="P6" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q6" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="R6" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="S6" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="T6" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="U6" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="V6" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="W6" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="X6" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="Y6" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="Z6" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="AA6" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="AB6" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC6" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="AD6" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="AE6" s="26" t="s">
+        <v>97</v>
+      </c>
+      <c r="AF6" s="26" t="s">
+        <v>98</v>
+      </c>
+      <c r="AG6" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="AH6" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="AI6" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="AJ6" s="26" t="s">
+        <v>102</v>
+      </c>
+      <c r="AK6" s="26" t="s">
+        <v>103</v>
+      </c>
+      <c r="AL6" s="26" t="s">
+        <v>104</v>
+      </c>
+      <c r="AM6" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="AN6" s="26" t="s">
+        <v>106</v>
+      </c>
+      <c r="AO6" s="26" t="s">
+        <v>107</v>
+      </c>
+      <c r="AP6" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="AQ6" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="AR6" s="26" t="s">
+        <v>110</v>
+      </c>
+      <c r="AS6" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="AT6" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="AU6" s="26" t="s">
+        <v>113</v>
+      </c>
+      <c r="AV6" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="AW6" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="AX6" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="AY6" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="AZ6" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="BA6" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="BB6" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="BC6" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="BD6" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="BE6" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="BF6" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="BG6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="BH6" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="BI6" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="BJ6" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="BK6" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="BL6" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="BM6" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="BN6" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="BO6" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="BP6" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="BQ6" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="BR6" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="BS6" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="BT6" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="BU6" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="BV6" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="BW6" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="BX6" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="BY6" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="BZ6" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="D6" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="H6" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="I6" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="J6" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="K6" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="L6" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="M6" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="N6" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="O6" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="P6" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="Q6" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="R6" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="S6" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="T6" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="U6" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="V6" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="W6" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="X6" s="11" t="s">
+      <c r="CA6" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="Y6" s="18" t="s">
+      <c r="CB6" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="Z6" s="11" t="s">
+      <c r="CC6" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="AA6" s="18" t="s">
+      <c r="CD6" s="11" t="s">
         <v>129</v>
-      </c>
-      <c r="AB6" s="11" t="s">
-        <v>130</v>
-      </c>
-      <c r="AC6" s="18" t="s">
-        <v>131</v>
-      </c>
-      <c r="AD6" s="25" t="s">
-        <v>132</v>
-      </c>
-      <c r="AE6" s="26" t="s">
-        <v>133</v>
-      </c>
-      <c r="AF6" s="26" t="s">
-        <v>134</v>
-      </c>
-      <c r="AG6" s="26" t="s">
-        <v>135</v>
-      </c>
-      <c r="AH6" s="26" t="s">
-        <v>136</v>
-      </c>
-      <c r="AI6" s="26" t="s">
-        <v>137</v>
-      </c>
-      <c r="AJ6" s="26" t="s">
-        <v>138</v>
-      </c>
-      <c r="AK6" s="26" t="s">
-        <v>139</v>
-      </c>
-      <c r="AL6" s="26" t="s">
-        <v>140</v>
-      </c>
-      <c r="AM6" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="AN6" s="26" t="s">
-        <v>142</v>
-      </c>
-      <c r="AO6" s="26" t="s">
-        <v>143</v>
-      </c>
-      <c r="AP6" s="26" t="s">
-        <v>144</v>
-      </c>
-      <c r="AQ6" s="26" t="s">
-        <v>145</v>
-      </c>
-      <c r="AR6" s="26" t="s">
-        <v>146</v>
-      </c>
-      <c r="AS6" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="AT6" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="AU6" s="26" t="s">
-        <v>149</v>
-      </c>
-      <c r="AV6" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="AW6" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="AX6" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="AY6" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="AZ6" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="BA6" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="BB6" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="BC6" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="BD6" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="BE6" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="BF6" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="BG6" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="BH6" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="BI6" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="BJ6" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="BK6" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="BL6" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="BM6" s="11" t="s">
-        <v>156</v>
-      </c>
-      <c r="BN6" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="BO6" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="BP6" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="BQ6" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="BR6" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="BS6" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="BT6" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="BU6" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="BV6" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="BW6" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="BX6" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="BY6" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="BZ6" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="CA6" s="11" t="s">
-        <v>162</v>
-      </c>
-      <c r="CB6" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="CC6" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="CD6" s="11" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="7" spans="1:82">
       <c r="A7" s="13" t="s">
-        <v>166</v>
+        <v>130</v>
       </c>
       <c r="B7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="C7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="D7" s="15" t="b">
         <v>1</v>
@@ -5545,28 +5298,28 @@
         <v>1</v>
       </c>
       <c r="F7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="G7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="H7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="I7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="J7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="K7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="L7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="M7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="N7" s="3">
         <v>1.1000000000000001</v>
@@ -5578,43 +5331,43 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="Q7" s="3" t="s" cm="1">
-        <v>168</v>
+        <v>132</v>
       </c>
       <c r="R7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="S7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="T7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="U7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="V7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="W7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="X7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="Y7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="Z7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="AA7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="AB7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="AC7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="AD7" s="27"/>
       <c r="AE7" s="27"/>
@@ -5635,7 +5388,7 @@
       <c r="AT7" s="27"/>
       <c r="AU7" s="27"/>
       <c r="AV7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="AW7" s="14">
         <v>1</v>
@@ -5647,55 +5400,55 @@
         <v>1</v>
       </c>
       <c r="AZ7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BA7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BB7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BC7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BD7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BE7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BF7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BG7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BH7" s="3" t="s" cm="1">
-        <v>168</v>
+        <v>132</v>
       </c>
       <c r="BI7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BJ7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BK7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BL7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BM7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BN7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BO7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BP7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BQ7" s="14">
         <v>1</v>
@@ -5704,16 +5457,16 @@
         <v>1</v>
       </c>
       <c r="BS7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BT7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="BU7" s="3">
         <v>1.1000000000000001</v>
       </c>
       <c r="BV7" s="3" t="s" cm="1">
-        <v>168</v>
+        <v>132</v>
       </c>
       <c r="BW7" s="3">
         <v>1.1000000000000001</v>
@@ -5734,18 +5487,18 @@
         <v>1</v>
       </c>
       <c r="CC7" s="3" t="s" cm="1">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="CD7" s="3" t="s">
-        <v>168</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:82" ht="23.25">
       <c r="B8" s="4" t="s">
-        <v>169</v>
+        <v>133</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>169</v>
+        <v>133</v>
       </c>
       <c r="D8" s="3" t="b">
         <v>1</v>
@@ -5754,25 +5507,25 @@
         <v>1</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>170</v>
+        <v>134</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>171</v>
+        <v>135</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>172</v>
+        <v>136</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>173</v>
+        <v>137</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>174</v>
+        <v>138</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>175</v>
+        <v>139</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>176</v>
+        <v>140</v>
       </c>
       <c r="N8" s="3">
         <v>1300</v>
@@ -5787,40 +5540,40 @@
         <v>2</v>
       </c>
       <c r="R8" s="3" t="s">
-        <v>177</v>
+        <v>141</v>
       </c>
       <c r="S8" s="4" t="s">
-        <v>178</v>
+        <v>142</v>
       </c>
       <c r="T8" s="4" t="s">
-        <v>179</v>
+        <v>143</v>
       </c>
       <c r="U8" s="4" t="s">
-        <v>180</v>
+        <v>144</v>
       </c>
       <c r="V8" s="4" t="s">
-        <v>181</v>
+        <v>145</v>
       </c>
       <c r="W8" s="4" t="s">
-        <v>182</v>
+        <v>146</v>
       </c>
       <c r="X8" s="4" t="s">
-        <v>183</v>
+        <v>147</v>
       </c>
       <c r="Y8" s="4" t="s">
-        <v>184</v>
+        <v>148</v>
       </c>
       <c r="Z8" s="4" t="s">
-        <v>185</v>
+        <v>149</v>
       </c>
       <c r="AA8" s="4" t="s">
-        <v>186</v>
+        <v>150</v>
       </c>
       <c r="AB8" s="4" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
       <c r="AC8" s="4" t="s">
-        <v>188</v>
+        <v>152</v>
       </c>
       <c r="AD8" s="27"/>
       <c r="AE8" s="27"/>
@@ -5847,31 +5600,31 @@
         <v>38434</v>
       </c>
       <c r="BB8" s="2" t="s">
-        <v>189</v>
+        <v>153</v>
       </c>
       <c r="BC8" s="6" t="s">
-        <v>190</v>
+        <v>154</v>
       </c>
       <c r="BD8" s="6" t="s">
-        <v>191</v>
+        <v>155</v>
       </c>
       <c r="BE8" s="4" t="s">
-        <v>192</v>
+        <v>156</v>
       </c>
       <c r="BG8" s="7" t="s">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="BH8" s="3">
         <v>100</v>
       </c>
       <c r="BL8" s="4" t="s">
-        <v>194</v>
+        <v>158</v>
       </c>
       <c r="BS8" s="4" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="BT8" s="4" t="s">
-        <v>196</v>
+        <v>160</v>
       </c>
       <c r="BU8" s="3">
         <v>0</v>

</xml_diff>